<commit_message>
Marca muda de RENOVA CELL para VitalRise (site, 28 idiomas, documentos, anúncios)
- Nome da marca, cupom (RENOVA10 → VITAL10) e endereço (vitalrise.vercel.app) em todo o
  projeto; flexões ajustadas em finlandês, estoniano e croata.
- A pasta projetos/renova-cell continua com o mesmo nome (é o Root Directory na Vercel).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013VVvDZDB6MGd8kjnX4E42S
</commit_message>
<xml_diff>
--- a/projetos/renova-cell/03-estrategia/metas-kpi.xlsx
+++ b/projetos/renova-cell/03-estrategia/metas-kpi.xlsx
@@ -934,7 +934,7 @@
     <row r="1" ht="17.35" customHeight="1" s="67">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>RENOVA CELL — Premissas do modelo (USD)</t>
+          <t>VitalRise — Premissas do modelo (USD)</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
     <row r="18" ht="15" customHeight="1" s="67">
       <c r="A18" s="71" t="inlineStr">
         <is>
-          <t>3. Cupom RENOVA10</t>
+          <t>3. Cupom VITAL10</t>
         </is>
       </c>
       <c r="B18" s="72" t="n"/>
@@ -1308,7 +1308,7 @@
     <row r="19" ht="28.5" customHeight="1" s="67">
       <c r="A19" s="73" t="inlineStr">
         <is>
-          <t>Desconto do cupom RENOVA10</t>
+          <t>Desconto do cupom VITAL10</t>
         </is>
       </c>
       <c r="B19" s="77" t="n">
@@ -2372,7 +2372,7 @@
     <row r="1" ht="17.35" customHeight="1" s="67">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>RENOVA CELL — Unit economics por comprador (USD)</t>
+          <t>VitalRise — Unit economics por comprador (USD)</t>
         </is>
       </c>
       <c r="F1" s="85" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="10" ht="15" customHeight="1" s="67">
       <c r="A10" s="73" t="inlineStr">
         <is>
-          <t>(−) Desconto do cupom RENOVA10</t>
+          <t>(−) Desconto do cupom VITAL10</t>
         </is>
       </c>
       <c r="B10" s="97">
@@ -3631,7 +3631,7 @@
     <row r="1" ht="17.35" customHeight="1" s="67">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>RENOVA CELL — Funil por 1.000 visitantes</t>
+          <t>VitalRise — Funil por 1.000 visitantes</t>
         </is>
       </c>
     </row>
@@ -4385,7 +4385,7 @@
     <row r="1" ht="17.35" customHeight="1" s="67">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>RENOVA CELL — KPIs do funil, metas e alertas</t>
+          <t>VitalRise — KPIs do funil, metas e alertas</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5578,7 @@
       </c>
       <c r="B27" s="110" t="inlineStr">
         <is>
-          <t>Uso do cupom RENOVA10</t>
+          <t>Uso do cupom VITAL10</t>
         </is>
       </c>
       <c r="C27" s="105" t="inlineStr">
@@ -5588,7 +5588,7 @@
       </c>
       <c r="D27" s="105" t="inlineStr">
         <is>
-          <t>Stripe: Checkout Sessions com promotion code RENOVA10 (total_details.amount_discount &gt; 0).</t>
+          <t>Stripe: Checkout Sessions com promotion code VITAL10 (total_details.amount_discount &gt; 0).</t>
         </is>
       </c>
       <c r="E27" s="105" t="inlineStr">
@@ -6030,6 +6030,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="67">
       <c r="A3" s="71" t="inlineStr">
         <is>
@@ -6178,7 +6179,7 @@
       </c>
       <c r="B16" s="73" t="inlineStr">
         <is>
-          <t>Divergência encontrada no código: o cupom RENOVA10 é criado sem applies_to, então o Stripe desconta também o order bump, mas o carrinho (CheckoutFlow.tsx) calcula o desconto só sobre o plano. A chave "O cupom também desconta o order bump?" (Premissas §3) segue o que o Stripe cobra.</t>
+          <t>Divergência encontrada no código: o cupom VITAL10 é criado sem applies_to, então o Stripe desconta também o order bump, mas o carrinho (CheckoutFlow.tsx) calcula o desconto só sobre o plano. A chave "O cupom também desconta o order bump?" (Premissas §3) segue o que o Stripe cobra.</t>
         </is>
       </c>
     </row>

</xml_diff>